<commit_message>
Add mtime file for controle_notas_07_julho.xlsx with timestamp
</commit_message>
<xml_diff>
--- a/planilhas_cache/METAS RJ.xlsx
+++ b/planilhas_cache/METAS RJ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Drives compartilhados\Off Trade\Campanhas e Metas\METAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4811FD8-36DA-437F-9271-2C14EFFE0214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{281261D9-C8C3-4C5B-9456-C91CD65A43CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{40673C59-61F7-4ACE-BE3C-88D4D3C2E782}"/>
   </bookViews>
@@ -868,12 +868,8 @@
       <c r="H2" s="3">
         <v>0.15</v>
       </c>
-      <c r="I2" s="4">
-        <v>1000</v>
-      </c>
-      <c r="J2" s="3">
-        <v>0.05</v>
-      </c>
+      <c r="I2" s="4"/>
+      <c r="J2" s="3"/>
       <c r="K2" s="5">
         <v>3</v>
       </c>
@@ -884,7 +880,7 @@
         <v>30</v>
       </c>
       <c r="N2" s="3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O2" s="7"/>
       <c r="P2" s="3"/>
@@ -924,12 +920,8 @@
       <c r="H3" s="3">
         <v>0.15</v>
       </c>
-      <c r="I3" s="4">
-        <v>500</v>
-      </c>
-      <c r="J3" s="3">
-        <v>0.05</v>
-      </c>
+      <c r="I3" s="4"/>
+      <c r="J3" s="3"/>
       <c r="K3" s="5">
         <v>3</v>
       </c>
@@ -940,7 +932,7 @@
         <v>100</v>
       </c>
       <c r="N3" s="3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O3" s="7"/>
       <c r="P3" s="3"/>
@@ -980,12 +972,8 @@
       <c r="H4" s="3">
         <v>0.1</v>
       </c>
-      <c r="I4" s="4">
-        <v>500</v>
-      </c>
-      <c r="J4" s="3">
-        <v>0.05</v>
-      </c>
+      <c r="I4" s="4"/>
+      <c r="J4" s="3"/>
       <c r="K4" s="5">
         <v>3</v>
       </c>
@@ -996,7 +984,7 @@
         <v>65</v>
       </c>
       <c r="N4" s="3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O4" s="7">
         <v>3</v>
@@ -1040,12 +1028,8 @@
       <c r="H5" s="3">
         <v>0.1</v>
       </c>
-      <c r="I5" s="4">
-        <v>1500</v>
-      </c>
-      <c r="J5" s="3">
-        <v>0.05</v>
-      </c>
+      <c r="I5" s="4"/>
+      <c r="J5" s="3"/>
       <c r="K5" s="5">
         <v>3</v>
       </c>
@@ -1056,7 +1040,7 @@
         <v>35</v>
       </c>
       <c r="N5" s="3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O5" s="7">
         <v>7</v>
@@ -1100,12 +1084,8 @@
       <c r="H6" s="3">
         <v>0.15</v>
       </c>
-      <c r="I6" s="4">
-        <v>1000</v>
-      </c>
-      <c r="J6" s="3">
-        <v>0.05</v>
-      </c>
+      <c r="I6" s="4"/>
+      <c r="J6" s="3"/>
       <c r="K6" s="5">
         <v>3</v>
       </c>
@@ -1116,7 +1096,7 @@
         <v>10</v>
       </c>
       <c r="N6" s="3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O6" s="7"/>
       <c r="P6" s="3"/>
@@ -1156,12 +1136,8 @@
       <c r="H7" s="3">
         <v>0.3</v>
       </c>
-      <c r="I7" s="4">
-        <v>1500</v>
-      </c>
-      <c r="J7" s="3">
-        <v>0</v>
-      </c>
+      <c r="I7" s="4"/>
+      <c r="J7" s="3"/>
       <c r="K7" s="5">
         <v>0</v>
       </c>
@@ -1212,12 +1188,8 @@
       <c r="H8" s="3">
         <v>0.1</v>
       </c>
-      <c r="I8" s="4">
-        <v>1500</v>
-      </c>
-      <c r="J8" s="3">
-        <v>0.05</v>
-      </c>
+      <c r="I8" s="4"/>
+      <c r="J8" s="3"/>
       <c r="K8" s="5">
         <v>4</v>
       </c>
@@ -1228,7 +1200,7 @@
         <v>50</v>
       </c>
       <c r="N8" s="3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O8" s="7">
         <v>7</v>
@@ -1272,12 +1244,8 @@
       <c r="H9" s="3">
         <v>0.1</v>
       </c>
-      <c r="I9" s="4">
-        <v>1500</v>
-      </c>
-      <c r="J9" s="3">
-        <v>0.05</v>
-      </c>
+      <c r="I9" s="4"/>
+      <c r="J9" s="3"/>
       <c r="K9" s="5">
         <v>4</v>
       </c>
@@ -1288,7 +1256,7 @@
         <v>50</v>
       </c>
       <c r="N9" s="3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O9" s="7">
         <v>7</v>
@@ -1332,12 +1300,8 @@
       <c r="H10" s="3">
         <v>0.15</v>
       </c>
-      <c r="I10" s="4">
-        <v>1000</v>
-      </c>
-      <c r="J10" s="3">
-        <v>0.05</v>
-      </c>
+      <c r="I10" s="4"/>
+      <c r="J10" s="3"/>
       <c r="K10" s="5">
         <v>3</v>
       </c>
@@ -1348,7 +1312,7 @@
         <v>45</v>
       </c>
       <c r="N10" s="3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O10" s="7"/>
       <c r="P10" s="3"/>
@@ -1388,12 +1352,8 @@
       <c r="H11" s="3">
         <v>0.1</v>
       </c>
-      <c r="I11" s="4">
-        <v>1500</v>
-      </c>
-      <c r="J11" s="3">
-        <v>0.05</v>
-      </c>
+      <c r="I11" s="4"/>
+      <c r="J11" s="3"/>
       <c r="K11" s="5">
         <v>4</v>
       </c>
@@ -1404,7 +1364,7 @@
         <v>40</v>
       </c>
       <c r="N11" s="3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O11" s="7">
         <v>7</v>
@@ -1448,12 +1408,8 @@
       <c r="H12" s="3">
         <v>0.1</v>
       </c>
-      <c r="I12" s="4">
-        <v>1500</v>
-      </c>
-      <c r="J12" s="3">
-        <v>0.05</v>
-      </c>
+      <c r="I12" s="4"/>
+      <c r="J12" s="3"/>
       <c r="K12" s="5">
         <v>3</v>
       </c>
@@ -1464,7 +1420,7 @@
         <v>33</v>
       </c>
       <c r="N12" s="3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O12" s="7">
         <v>7</v>
@@ -1504,9 +1460,7 @@
         <v>60000</v>
       </c>
       <c r="H13" s="3"/>
-      <c r="I13" s="4">
-        <v>0</v>
-      </c>
+      <c r="I13" s="4"/>
       <c r="J13" s="3"/>
       <c r="K13" s="5">
         <v>3</v>
@@ -1554,12 +1508,8 @@
       <c r="H14" s="3">
         <v>0.05</v>
       </c>
-      <c r="I14" s="2">
-        <v>500</v>
-      </c>
-      <c r="J14" s="3">
-        <v>0.05</v>
-      </c>
+      <c r="I14" s="2"/>
+      <c r="J14" s="3"/>
       <c r="K14" s="5">
         <v>4</v>
       </c>
@@ -1570,7 +1520,7 @@
         <v>70</v>
       </c>
       <c r="N14" s="3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O14" s="8">
         <v>22</v>
@@ -1626,12 +1576,8 @@
       <c r="H15" s="3">
         <v>0.05</v>
       </c>
-      <c r="I15" s="2">
-        <v>500</v>
-      </c>
-      <c r="J15" s="3">
-        <v>0.05</v>
-      </c>
+      <c r="I15" s="2"/>
+      <c r="J15" s="3"/>
       <c r="K15" s="5">
         <v>3</v>
       </c>
@@ -1642,7 +1588,7 @@
         <v>70</v>
       </c>
       <c r="N15" s="3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O15" s="8">
         <v>22</v>
@@ -1698,12 +1644,8 @@
       <c r="H16" s="3">
         <v>0.05</v>
       </c>
-      <c r="I16" s="2">
-        <v>500</v>
-      </c>
-      <c r="J16" s="3">
-        <v>0.05</v>
-      </c>
+      <c r="I16" s="2"/>
+      <c r="J16" s="3"/>
       <c r="K16" s="5">
         <v>4</v>
       </c>
@@ -1714,7 +1656,7 @@
         <v>50</v>
       </c>
       <c r="N16" s="3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O16" s="8">
         <v>14</v>
@@ -1770,12 +1712,8 @@
       <c r="H17" s="3">
         <v>0.1</v>
       </c>
-      <c r="I17" s="2">
-        <v>500</v>
-      </c>
-      <c r="J17" s="3">
-        <v>0.05</v>
-      </c>
+      <c r="I17" s="2"/>
+      <c r="J17" s="3"/>
       <c r="K17" s="5">
         <v>3</v>
       </c>
@@ -1786,7 +1724,7 @@
         <v>50</v>
       </c>
       <c r="N17" s="3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O17" s="8">
         <v>10</v>

</xml_diff>

<commit_message>
Atualiza timestamps de arquivos de planilhas e modifica dados de autenticação de vendedores
</commit_message>
<xml_diff>
--- a/planilhas_cache/METAS RJ.xlsx
+++ b/planilhas_cache/METAS RJ.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Drives compartilhados\Off Trade\Campanhas e Metas\METAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{281261D9-C8C3-4C5B-9456-C91CD65A43CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B55CF1-E6C1-4AB4-8314-EB94C01CE03A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{40673C59-61F7-4ACE-BE3C-88D4D3C2E782}"/>
   </bookViews>
@@ -31,15 +31,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="66">
   <si>
     <t>VENDEDOR</t>
   </si>
@@ -216,6 +213,27 @@
   </si>
   <si>
     <t>DANIELLE MOURA</t>
+  </si>
+  <si>
+    <t>IVANILDO MAIA - OFF TRADE</t>
+  </si>
+  <si>
+    <t>META FATURAMENTO PERNOD</t>
+  </si>
+  <si>
+    <t>PESO FATURAMENTO PERNOD</t>
+  </si>
+  <si>
+    <t>META FATURAMENTO HOB + AZEITE</t>
+  </si>
+  <si>
+    <t>PESO FATURAMENTO HOB + AZEITE</t>
+  </si>
+  <si>
+    <t>META POSITIVAÇÃO ESSENZA+HOB</t>
+  </si>
+  <si>
+    <t>PESO POSITIVAÇÃO ESSENZA+HOB</t>
   </si>
 </sst>
 </file>
@@ -226,7 +244,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -277,6 +295,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -298,7 +323,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -321,13 +346,265 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color theme="2"/>
+      </left>
+      <right style="medium">
+        <color theme="2"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="2"/>
+      </left>
+      <right style="medium">
+        <color theme="2"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="2"/>
+      </left>
+      <right style="medium">
+        <color theme="2"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="0" tint="-0.499984740745262"/>
+      </left>
+      <right style="medium">
+        <color theme="2"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="0" tint="-0.499984740745262"/>
+      </left>
+      <right style="medium">
+        <color theme="2"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color theme="2"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color theme="2"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top style="thin">
+        <color theme="2"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="2"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="2"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top style="thin">
+        <color theme="2"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="2"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="2"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="44" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -414,6 +691,99 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="2" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -421,7 +791,663 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="34">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="22" formatCode="mmm/yy"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -434,10 +1460,51 @@
 </styleSheet>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FF22F818-041C-4A47-BAD6-A18C548D390B}" name="Tabela2" displayName="Tabela2" ref="A1:AF45" totalsRowShown="0" dataDxfId="1" tableBorderDxfId="33">
+  <autoFilter ref="A1:AF45" xr:uid="{FF22F818-041C-4A47-BAD6-A18C548D390B}"/>
+  <tableColumns count="32">
+    <tableColumn id="1" xr3:uid="{94196E2A-EF93-427A-92BE-CAFE797C153A}" name="CONTRATO" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{0033F0AB-E800-4A63-9A0F-3F37D56071ED}" name="VENDEDOR" dataDxfId="31" dataCellStyle="Porcentagem"/>
+    <tableColumn id="3" xr3:uid="{550D04B9-6CA2-4AE6-8C2C-F63D358ACC13}" name="RCA" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{46A57AE2-12D9-4C02-8647-113FFD6665E5}" name="MÊS" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{F1D9D24D-90FD-412D-906A-C83471538538}" name="META FATURAMENTO" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{88ADA9E4-4A63-4F71-B6C1-E2EADAB30711}" name="PESO FATURAMENTO" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{796CFDC2-1174-46D2-8FAD-7941CB5234D4}" name="META FATURAMENTO CASTAS" dataDxfId="27"/>
+    <tableColumn id="8" xr3:uid="{107F2C71-9B78-4DBB-9071-31CF3985E967}" name="PESO FATURAMENTO CASTAS" dataDxfId="26"/>
+    <tableColumn id="9" xr3:uid="{D4EF19D6-365B-4934-8799-B133BDF0E8EB}" name="META FATURAMENTO AZEITE" dataDxfId="25"/>
+    <tableColumn id="10" xr3:uid="{3C1228DF-3AD5-4CB1-B6A3-A05D9A7B1282}" name="PESO FATURAMENTO AZEITE" dataDxfId="24"/>
+    <tableColumn id="11" xr3:uid="{D983D94B-C943-4904-AE07-24F70785FBFF}" name="META POSITIVAÇÃO HOB + AZEITE" dataDxfId="23"/>
+    <tableColumn id="12" xr3:uid="{93E7AA27-EA98-4AB3-8369-440936701C16}" name="PESO POSITIVAÇÃO HOB + AZEITE" dataDxfId="22"/>
+    <tableColumn id="13" xr3:uid="{57E4A5E0-9648-44FC-BDBE-51833B1FCBE3}" name="META POSITIVAÇÃO" dataDxfId="21"/>
+    <tableColumn id="14" xr3:uid="{9A233F5A-DAAA-4411-9EE5-937E6810301F}" name="PESO POSITIVAÇÃO" dataDxfId="20"/>
+    <tableColumn id="15" xr3:uid="{5B674825-C848-4FE0-9E94-0718BF70F9EA}" name="META POSITIVAÇÃO RECKIT" dataDxfId="19"/>
+    <tableColumn id="16" xr3:uid="{1C062D5A-AA84-4F6A-9217-81635F0D3B15}" name="PESO POSITIVAÇÃO RECKIT" dataDxfId="18"/>
+    <tableColumn id="17" xr3:uid="{E14DDDB6-B770-487C-BD25-F3710535C37A}" name="META POSITIVAÇÃO TIAL" dataDxfId="17"/>
+    <tableColumn id="18" xr3:uid="{C03A3836-ABA4-41E8-9013-0D52B8BFEF8C}" name="PESO POSITIVAÇÃO TIAL" dataDxfId="16"/>
+    <tableColumn id="19" xr3:uid="{1B39F49C-DC43-4B74-B3D0-0C90B5B46334}" name="META POSITIVAÇÃO TATUZINHO" dataDxfId="15"/>
+    <tableColumn id="20" xr3:uid="{4AE519C7-AACA-4C84-8C01-42F4D72DF594}" name="PESO POSITIVAÇÃO TATUZINHO" dataDxfId="14"/>
+    <tableColumn id="21" xr3:uid="{63E60540-4C47-44B9-994B-38355CC42EF8}" name="META POSITIVAÇÃO RED BULL" dataDxfId="13"/>
+    <tableColumn id="22" xr3:uid="{94108FCC-48D1-4D71-A4F5-B0B2492E529A}" name="PESO POSITIVAÇÃO RED BULL" dataDxfId="12"/>
+    <tableColumn id="23" xr3:uid="{867D4BD1-AFF0-464D-85ED-DEBF82C15687}" name="META POSITIVAÇÃO PINATTI" dataDxfId="11"/>
+    <tableColumn id="24" xr3:uid="{C644C171-0011-444B-B3F6-481E165C42F1}" name="PESO POSITIVAÇÃO PINATTI" dataDxfId="10"/>
+    <tableColumn id="25" xr3:uid="{5D1F0FF6-5D1B-4004-9F38-EBD7339B37B8}" name="META POSITIVAÇÃO ESSENZA" dataDxfId="9"/>
+    <tableColumn id="26" xr3:uid="{E812DE08-D864-4479-B8F7-BE7ED72A1C5D}" name="PESO POSITIVAÇÃO ESSENZA" dataDxfId="8"/>
+    <tableColumn id="27" xr3:uid="{F33E0E05-C616-4D77-8716-8D9A891CEA56}" name="META FATURAMENTO PERNOD" dataDxfId="7"/>
+    <tableColumn id="28" xr3:uid="{3C0B200C-9CF2-4AD8-AF4C-97A32B262CB6}" name="PESO FATURAMENTO PERNOD" dataDxfId="6"/>
+    <tableColumn id="29" xr3:uid="{85C3AFCE-64C8-4A21-8584-0F285733B6CD}" name="META FATURAMENTO HOB + AZEITE" dataDxfId="5"/>
+    <tableColumn id="30" xr3:uid="{613F3555-4481-400A-9B43-1DBD98888D67}" name="PESO FATURAMENTO HOB + AZEITE" dataDxfId="4"/>
+    <tableColumn id="31" xr3:uid="{45BDBA07-5EC9-4BD4-A31B-064F071EEC2C}" name="META POSITIVAÇÃO ESSENZA+HOB" dataDxfId="3"/>
+    <tableColumn id="32" xr3:uid="{91748D3D-C321-4344-B927-5E0F477576C2}" name="PESO POSITIVAÇÃO ESSENZA+HOB" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -475,7 +1542,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -581,7 +1648,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -723,7 +1790,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -731,46 +1798,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB96CD6D-1F44-4A59-BB02-A23ABD5F87F6}">
-  <dimension ref="A1:Z23"/>
+  <dimension ref="A1:AF45"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.109375" style="30" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19" style="30" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.21875" style="30" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.88671875" style="65" customWidth="1"/>
     <col min="4" max="4" width="6.33203125" style="30" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.5546875" style="30" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.109375" style="30" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25" style="30" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.5546875" style="30" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.33203125" style="30" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.88671875" style="30" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="28.44140625" style="30" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="28" style="30" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17" style="30" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.5546875" style="30" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="23.109375" style="30" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="22.6640625" style="30" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.88671875" style="30" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.44140625" style="30" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="27.109375" style="30" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="26.6640625" style="30" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="25.21875" style="30" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="24.77734375" style="30" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="23.88671875" style="30" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="23.44140625" style="30" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="24.44140625" style="30" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="24" style="30" bestFit="1" customWidth="1"/>
-    <col min="27" max="16384" width="8.88671875" style="30"/>
+    <col min="5" max="5" width="19.44140625" style="30" customWidth="1"/>
+    <col min="6" max="6" width="19" style="30" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" style="30" customWidth="1"/>
+    <col min="8" max="9" width="25.109375" style="30" customWidth="1"/>
+    <col min="10" max="10" width="24.5546875" style="30" customWidth="1"/>
+    <col min="11" max="11" width="28.6640625" style="30" customWidth="1"/>
+    <col min="12" max="12" width="28.109375" style="30" customWidth="1"/>
+    <col min="13" max="13" width="17.88671875" style="30" customWidth="1"/>
+    <col min="14" max="14" width="17.33203125" style="30" customWidth="1"/>
+    <col min="15" max="15" width="23.6640625" style="30" customWidth="1"/>
+    <col min="16" max="16" width="23.109375" style="30" customWidth="1"/>
+    <col min="17" max="17" width="21.5546875" style="30" customWidth="1"/>
+    <col min="18" max="18" width="21" style="30" customWidth="1"/>
+    <col min="19" max="19" width="27.33203125" style="30" customWidth="1"/>
+    <col min="20" max="20" width="26.77734375" style="30" customWidth="1"/>
+    <col min="21" max="21" width="25.6640625" style="30" customWidth="1"/>
+    <col min="22" max="22" width="25.109375" style="30" customWidth="1"/>
+    <col min="23" max="23" width="24.33203125" style="30" customWidth="1"/>
+    <col min="24" max="24" width="23.77734375" style="30" customWidth="1"/>
+    <col min="25" max="25" width="25.109375" style="30" customWidth="1"/>
+    <col min="26" max="26" width="24.5546875" style="30" customWidth="1"/>
+    <col min="27" max="27" width="28.21875" style="30" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="27.77734375" style="30" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="32.21875" style="30" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="31.77734375" style="30" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="31.33203125" style="30" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="30.88671875" style="30" bestFit="1" customWidth="1"/>
+    <col min="33" max="16384" width="8.88671875" style="30"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A1" s="61" t="s">
         <v>45</v>
       </c>
       <c r="B1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="63" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="11" t="s">
@@ -842,15 +1914,33 @@
       <c r="Z1" s="11" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="2" spans="1:26" s="31" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
+      <c r="AA1" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="AB1" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="AC1" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="AD1" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="AE1" s="52" t="s">
+        <v>64</v>
+      </c>
+      <c r="AF1" s="52" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:32" s="31" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="62" t="s">
         <v>48</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="14">
+      <c r="C2" s="64">
         <v>275</v>
       </c>
       <c r="D2" s="15">
@@ -895,14 +1985,14 @@
       <c r="Y2" s="14"/>
       <c r="Z2" s="14"/>
     </row>
-    <row r="3" spans="1:26" s="31" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+    <row r="3" spans="1:32" s="31" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="62" t="s">
         <v>48</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="14">
+      <c r="C3" s="64">
         <v>156</v>
       </c>
       <c r="D3" s="15">
@@ -947,14 +2037,14 @@
       <c r="Y3" s="14"/>
       <c r="Z3" s="14"/>
     </row>
-    <row r="4" spans="1:26" s="31" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
+    <row r="4" spans="1:32" s="31" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="62" t="s">
         <v>48</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="14">
+      <c r="C4" s="64">
         <v>412</v>
       </c>
       <c r="D4" s="15">
@@ -1003,14 +2093,14 @@
       <c r="Y4" s="14"/>
       <c r="Z4" s="14"/>
     </row>
-    <row r="5" spans="1:26" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="13" t="s">
+    <row r="5" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="62" t="s">
         <v>48</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="14">
+      <c r="C5" s="64">
         <v>153</v>
       </c>
       <c r="D5" s="15">
@@ -1059,14 +2149,14 @@
       <c r="Y5" s="16"/>
       <c r="Z5" s="16"/>
     </row>
-    <row r="6" spans="1:26" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="13" t="s">
+    <row r="6" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="62" t="s">
         <v>48</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="14">
+      <c r="C6" s="64">
         <v>158</v>
       </c>
       <c r="D6" s="15">
@@ -1111,14 +2201,14 @@
       <c r="Y6" s="16"/>
       <c r="Z6" s="16"/>
     </row>
-    <row r="7" spans="1:26" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
+    <row r="7" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="62" t="s">
         <v>48</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="64">
         <v>238</v>
       </c>
       <c r="D7" s="15">
@@ -1163,14 +2253,14 @@
       <c r="Y7" s="16"/>
       <c r="Z7" s="16"/>
     </row>
-    <row r="8" spans="1:26" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="13" t="s">
+    <row r="8" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="62" t="s">
         <v>48</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="64">
         <v>419</v>
       </c>
       <c r="D8" s="15">
@@ -1219,14 +2309,14 @@
       <c r="Y8" s="16"/>
       <c r="Z8" s="16"/>
     </row>
-    <row r="9" spans="1:26" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="13" t="s">
+    <row r="9" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="62" t="s">
         <v>48</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="64">
         <v>144</v>
       </c>
       <c r="D9" s="15">
@@ -1275,14 +2365,14 @@
       <c r="Y9" s="16"/>
       <c r="Z9" s="16"/>
     </row>
-    <row r="10" spans="1:26" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="13" t="s">
+    <row r="10" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="62" t="s">
         <v>48</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="64">
         <v>450</v>
       </c>
       <c r="D10" s="15">
@@ -1327,14 +2417,14 @@
       <c r="Y10" s="16"/>
       <c r="Z10" s="16"/>
     </row>
-    <row r="11" spans="1:26" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="13" t="s">
+    <row r="11" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="62" t="s">
         <v>47</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="64">
         <v>417</v>
       </c>
       <c r="D11" s="15">
@@ -1383,14 +2473,14 @@
       <c r="Y11" s="16"/>
       <c r="Z11" s="16"/>
     </row>
-    <row r="12" spans="1:26" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="13" t="s">
+    <row r="12" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="62" t="s">
         <v>47</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="64">
         <v>439</v>
       </c>
       <c r="D12" s="15">
@@ -1439,14 +2529,14 @@
       <c r="Y12" s="16"/>
       <c r="Z12" s="16"/>
     </row>
-    <row r="13" spans="1:26" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="13" t="s">
+    <row r="13" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="62" t="s">
         <v>50</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="14">
+      <c r="C13" s="64">
         <v>420</v>
       </c>
       <c r="D13" s="15">
@@ -1483,14 +2573,14 @@
       <c r="Y13" s="16"/>
       <c r="Z13" s="16"/>
     </row>
-    <row r="14" spans="1:26" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="13" t="s">
+    <row r="14" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="62" t="s">
         <v>49</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="64">
         <v>431</v>
       </c>
       <c r="D14" s="15">
@@ -1551,14 +2641,14 @@
       <c r="Y14" s="16"/>
       <c r="Z14" s="16"/>
     </row>
-    <row r="15" spans="1:26" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="13" t="s">
+    <row r="15" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="62" t="s">
         <v>49</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="64">
         <v>379</v>
       </c>
       <c r="D15" s="15">
@@ -1619,14 +2709,14 @@
       <c r="Y15" s="16"/>
       <c r="Z15" s="16"/>
     </row>
-    <row r="16" spans="1:26" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="13" t="s">
+    <row r="16" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="62" t="s">
         <v>49</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="64">
         <v>471</v>
       </c>
       <c r="D16" s="15">
@@ -1687,14 +2777,14 @@
       <c r="Y16" s="16"/>
       <c r="Z16" s="16"/>
     </row>
-    <row r="17" spans="1:26" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="13" t="s">
+    <row r="17" spans="1:30" s="32" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="62" t="s">
         <v>49</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="14">
+      <c r="C17" s="64">
         <v>378</v>
       </c>
       <c r="D17" s="15">
@@ -1759,14 +2849,14 @@
       <c r="Y17" s="16"/>
       <c r="Z17" s="16"/>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A18" s="13" t="s">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A18" s="62" t="s">
         <v>48</v>
       </c>
       <c r="B18" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="13">
+      <c r="C18" s="64">
         <v>91</v>
       </c>
       <c r="D18" s="15">
@@ -1795,14 +2885,14 @@
       <c r="Y18" s="13"/>
       <c r="Z18" s="13"/>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A19" s="13" t="s">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A19" s="62" t="s">
         <v>47</v>
       </c>
       <c r="B19" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="13">
+      <c r="C19" s="64">
         <v>446</v>
       </c>
       <c r="D19" s="15">
@@ -1831,14 +2921,14 @@
       <c r="Y19" s="13"/>
       <c r="Z19" s="13"/>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A20" s="13" t="s">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A20" s="62" t="s">
         <v>48</v>
       </c>
       <c r="B20" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="13">
+      <c r="C20" s="64">
         <v>174</v>
       </c>
       <c r="D20" s="15">
@@ -1867,14 +2957,14 @@
       <c r="Y20" s="13"/>
       <c r="Z20" s="13"/>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A21" s="13" t="s">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A21" s="62" t="s">
         <v>46</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="13">
+      <c r="C21" s="64">
         <v>159</v>
       </c>
       <c r="D21" s="15">
@@ -1903,14 +2993,14 @@
       <c r="Y21" s="13"/>
       <c r="Z21" s="13"/>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A22" s="13" t="s">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A22" s="62" t="s">
         <v>46</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="13">
+      <c r="C22" s="64">
         <v>155</v>
       </c>
       <c r="D22" s="15">
@@ -1939,14 +3029,14 @@
       <c r="Y22" s="13"/>
       <c r="Z22" s="13"/>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A23" s="13" t="s">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A23" s="62" t="s">
         <v>46</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="13">
+      <c r="C23" s="64">
         <v>241</v>
       </c>
       <c r="D23" s="15">
@@ -1975,9 +3065,826 @@
       <c r="Y23" s="13"/>
       <c r="Z23" s="13"/>
     </row>
+    <row r="24" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C24" s="64">
+        <v>275</v>
+      </c>
+      <c r="D24" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E24" s="34">
+        <v>345000</v>
+      </c>
+      <c r="F24" s="37">
+        <v>0.7</v>
+      </c>
+      <c r="G24" s="34">
+        <v>44000</v>
+      </c>
+      <c r="H24" s="42">
+        <v>0.1</v>
+      </c>
+      <c r="M24" s="45">
+        <v>30</v>
+      </c>
+      <c r="N24" s="49">
+        <v>0.1</v>
+      </c>
+      <c r="AA24" s="34">
+        <v>25000</v>
+      </c>
+      <c r="AB24" s="37">
+        <v>0.05</v>
+      </c>
+      <c r="AC24" s="43">
+        <v>9500</v>
+      </c>
+      <c r="AD24" s="37">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="25" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="64">
+        <v>156</v>
+      </c>
+      <c r="D25" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E25" s="34">
+        <v>90000</v>
+      </c>
+      <c r="F25" s="37">
+        <v>0.7</v>
+      </c>
+      <c r="G25" s="34">
+        <v>9000</v>
+      </c>
+      <c r="H25" s="42">
+        <v>0.1</v>
+      </c>
+      <c r="M25" s="45">
+        <v>70</v>
+      </c>
+      <c r="N25" s="49">
+        <v>0.1</v>
+      </c>
+      <c r="AA25" s="34">
+        <v>7000</v>
+      </c>
+      <c r="AB25" s="37">
+        <v>0.05</v>
+      </c>
+      <c r="AC25" s="43">
+        <v>1000</v>
+      </c>
+      <c r="AD25" s="37">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="26" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C26" s="64">
+        <v>412</v>
+      </c>
+      <c r="D26" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E26" s="34">
+        <v>150000</v>
+      </c>
+      <c r="F26" s="37">
+        <v>0.7</v>
+      </c>
+      <c r="G26" s="34">
+        <v>9000</v>
+      </c>
+      <c r="H26" s="42">
+        <v>0.1</v>
+      </c>
+      <c r="M26" s="45">
+        <v>50</v>
+      </c>
+      <c r="N26" s="49">
+        <v>0.1</v>
+      </c>
+      <c r="AA26" s="34">
+        <v>7000</v>
+      </c>
+      <c r="AB26" s="37">
+        <v>0.05</v>
+      </c>
+      <c r="AC26" s="43">
+        <v>1500</v>
+      </c>
+      <c r="AD26" s="37">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="27" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" s="64">
+        <v>153</v>
+      </c>
+      <c r="D27" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E27" s="34">
+        <v>190000</v>
+      </c>
+      <c r="F27" s="37">
+        <v>0.7</v>
+      </c>
+      <c r="G27" s="34">
+        <v>10000</v>
+      </c>
+      <c r="H27" s="42">
+        <v>0.1</v>
+      </c>
+      <c r="M27" s="45">
+        <v>50</v>
+      </c>
+      <c r="N27" s="49">
+        <v>0.1</v>
+      </c>
+      <c r="AA27" s="34">
+        <v>25000</v>
+      </c>
+      <c r="AB27" s="37">
+        <v>0.05</v>
+      </c>
+      <c r="AC27" s="43">
+        <v>1500</v>
+      </c>
+      <c r="AD27" s="37">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="28" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="64">
+        <v>158</v>
+      </c>
+      <c r="D28" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E28" s="34">
+        <v>450000</v>
+      </c>
+      <c r="F28" s="37">
+        <v>0.7</v>
+      </c>
+      <c r="G28" s="34">
+        <v>12000</v>
+      </c>
+      <c r="H28" s="42">
+        <v>0.1</v>
+      </c>
+      <c r="M28" s="45">
+        <v>10</v>
+      </c>
+      <c r="N28" s="49">
+        <v>0.1</v>
+      </c>
+      <c r="AA28" s="34">
+        <v>20000</v>
+      </c>
+      <c r="AB28" s="37">
+        <v>0.05</v>
+      </c>
+      <c r="AC28" s="43">
+        <v>1500</v>
+      </c>
+      <c r="AD28" s="37">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="29" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C29" s="64">
+        <v>238</v>
+      </c>
+      <c r="D29" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E29" s="34">
+        <v>150000</v>
+      </c>
+      <c r="F29" s="37">
+        <v>0.8</v>
+      </c>
+      <c r="G29" s="34">
+        <v>3000</v>
+      </c>
+      <c r="H29" s="42">
+        <v>0.1</v>
+      </c>
+      <c r="M29" s="45">
+        <v>1</v>
+      </c>
+      <c r="N29" s="49">
+        <v>0.1</v>
+      </c>
+      <c r="AA29" s="34">
+        <v>0</v>
+      </c>
+      <c r="AB29" s="37"/>
+      <c r="AC29" s="43">
+        <v>0</v>
+      </c>
+      <c r="AD29" s="37"/>
+    </row>
+    <row r="30" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" s="64">
+        <v>419</v>
+      </c>
+      <c r="D30" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E30" s="34">
+        <v>130000</v>
+      </c>
+      <c r="F30" s="37">
+        <v>0.7</v>
+      </c>
+      <c r="G30" s="34">
+        <v>10000</v>
+      </c>
+      <c r="H30" s="42">
+        <v>0.1</v>
+      </c>
+      <c r="M30" s="45">
+        <v>50</v>
+      </c>
+      <c r="N30" s="49">
+        <v>0.1</v>
+      </c>
+      <c r="AA30" s="34">
+        <v>20000</v>
+      </c>
+      <c r="AB30" s="37">
+        <v>0.05</v>
+      </c>
+      <c r="AC30" s="43">
+        <v>1500</v>
+      </c>
+      <c r="AD30" s="37">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="31" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" s="64">
+        <v>144</v>
+      </c>
+      <c r="D31" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E31" s="34">
+        <v>190000</v>
+      </c>
+      <c r="F31" s="37">
+        <v>0.7</v>
+      </c>
+      <c r="G31" s="34">
+        <v>10000</v>
+      </c>
+      <c r="H31" s="42">
+        <v>0.1</v>
+      </c>
+      <c r="M31" s="45">
+        <v>35</v>
+      </c>
+      <c r="N31" s="49">
+        <v>0.1</v>
+      </c>
+      <c r="AA31" s="34">
+        <v>30000</v>
+      </c>
+      <c r="AB31" s="37">
+        <v>0.05</v>
+      </c>
+      <c r="AC31" s="43">
+        <v>1500</v>
+      </c>
+      <c r="AD31" s="37">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="32" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C32" s="64">
+        <v>450</v>
+      </c>
+      <c r="D32" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E32" s="34">
+        <v>250000</v>
+      </c>
+      <c r="F32" s="37">
+        <v>0.7</v>
+      </c>
+      <c r="G32" s="34">
+        <v>10000</v>
+      </c>
+      <c r="H32" s="42">
+        <v>0.1</v>
+      </c>
+      <c r="M32" s="45">
+        <v>45</v>
+      </c>
+      <c r="N32" s="49">
+        <v>0.1</v>
+      </c>
+      <c r="AA32" s="34">
+        <v>30000</v>
+      </c>
+      <c r="AB32" s="37">
+        <v>0.05</v>
+      </c>
+      <c r="AC32" s="43">
+        <v>1500</v>
+      </c>
+      <c r="AD32" s="37">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="33" spans="1:32" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="62" t="s">
+        <v>47</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C33" s="64">
+        <v>439</v>
+      </c>
+      <c r="D33" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E33" s="34">
+        <v>450000</v>
+      </c>
+      <c r="F33" s="37">
+        <v>0.7</v>
+      </c>
+      <c r="G33" s="34">
+        <v>10000</v>
+      </c>
+      <c r="H33" s="42">
+        <v>0.1</v>
+      </c>
+      <c r="M33" s="46">
+        <v>50</v>
+      </c>
+      <c r="N33" s="49">
+        <v>0.1</v>
+      </c>
+      <c r="AA33" s="34">
+        <v>50000</v>
+      </c>
+      <c r="AB33" s="37">
+        <v>0.05</v>
+      </c>
+      <c r="AC33" s="43">
+        <v>1500</v>
+      </c>
+      <c r="AD33" s="37">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="34" spans="1:32" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="62" t="s">
+        <v>50</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" s="64">
+        <v>420</v>
+      </c>
+      <c r="D34" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E34" s="34">
+        <v>300000</v>
+      </c>
+      <c r="F34" s="37"/>
+      <c r="G34" s="35">
+        <v>60000</v>
+      </c>
+      <c r="M34" s="45">
+        <v>1</v>
+      </c>
+      <c r="N34" s="49"/>
+      <c r="AA34" s="34">
+        <v>350000</v>
+      </c>
+      <c r="AB34" s="37"/>
+      <c r="AC34" s="43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A35" s="62" t="s">
+        <v>47</v>
+      </c>
+      <c r="B35" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="C35" s="65">
+        <v>460</v>
+      </c>
+      <c r="D35" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E35" s="35">
+        <v>30000</v>
+      </c>
+      <c r="F35" s="38"/>
+      <c r="G35" s="41">
+        <v>1000</v>
+      </c>
+      <c r="M35" s="45">
+        <v>15</v>
+      </c>
+      <c r="N35" s="49"/>
+      <c r="AA35" s="35">
+        <v>24000</v>
+      </c>
+      <c r="AB35" s="38"/>
+      <c r="AC35" s="41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:32" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="62" t="s">
+        <v>49</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C36" s="64">
+        <v>431</v>
+      </c>
+      <c r="D36" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E36" s="36">
+        <v>65000</v>
+      </c>
+      <c r="F36" s="39">
+        <v>0.1</v>
+      </c>
+      <c r="G36" s="36">
+        <v>3000</v>
+      </c>
+      <c r="M36" s="47">
+        <v>70</v>
+      </c>
+      <c r="N36" s="50">
+        <v>0.7</v>
+      </c>
+      <c r="Q36" s="8">
+        <v>12</v>
+      </c>
+      <c r="R36" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="S36" s="54">
+        <v>15</v>
+      </c>
+      <c r="T36" s="59">
+        <v>0.05</v>
+      </c>
+      <c r="AA36" s="36">
+        <v>3000</v>
+      </c>
+      <c r="AB36" s="39">
+        <v>0.05</v>
+      </c>
+      <c r="AC36" s="44">
+        <v>1000</v>
+      </c>
+      <c r="AE36" s="53">
+        <v>0.05</v>
+      </c>
+      <c r="AF36" s="54">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:32" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="62" t="s">
+        <v>49</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C37" s="64">
+        <v>379</v>
+      </c>
+      <c r="D37" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E37" s="34">
+        <v>80000</v>
+      </c>
+      <c r="F37" s="37">
+        <v>0.1</v>
+      </c>
+      <c r="G37" s="34">
+        <v>3000</v>
+      </c>
+      <c r="M37" s="48">
+        <v>70</v>
+      </c>
+      <c r="N37" s="51">
+        <v>0.7</v>
+      </c>
+      <c r="Q37" s="8">
+        <v>12</v>
+      </c>
+      <c r="R37" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="S37" s="58">
+        <v>15</v>
+      </c>
+      <c r="T37" s="57">
+        <v>0.05</v>
+      </c>
+      <c r="AA37" s="34">
+        <v>3000</v>
+      </c>
+      <c r="AB37" s="37">
+        <v>0.05</v>
+      </c>
+      <c r="AC37" s="44">
+        <v>1000</v>
+      </c>
+      <c r="AE37" s="55">
+        <v>0.05</v>
+      </c>
+      <c r="AF37" s="56">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:32" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="62" t="s">
+        <v>49</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C38" s="64">
+        <v>471</v>
+      </c>
+      <c r="D38" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E38" s="34">
+        <v>65000</v>
+      </c>
+      <c r="F38" s="37">
+        <v>0.1</v>
+      </c>
+      <c r="G38" s="34">
+        <v>3000</v>
+      </c>
+      <c r="M38" s="48">
+        <v>50</v>
+      </c>
+      <c r="N38" s="51">
+        <v>0.7</v>
+      </c>
+      <c r="Q38" s="8">
+        <v>12</v>
+      </c>
+      <c r="R38" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="S38" s="58">
+        <v>15</v>
+      </c>
+      <c r="T38" s="57">
+        <v>0.05</v>
+      </c>
+      <c r="AA38" s="34">
+        <v>3000</v>
+      </c>
+      <c r="AB38" s="37">
+        <v>0.05</v>
+      </c>
+      <c r="AC38" s="44">
+        <v>1000</v>
+      </c>
+      <c r="AE38" s="57">
+        <v>0.05</v>
+      </c>
+      <c r="AF38" s="46">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:32" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="62" t="s">
+        <v>49</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" s="64">
+        <v>378</v>
+      </c>
+      <c r="D39" s="33">
+        <v>46204</v>
+      </c>
+      <c r="E39" s="34">
+        <v>65000</v>
+      </c>
+      <c r="F39" s="40">
+        <v>0.1</v>
+      </c>
+      <c r="G39" s="34">
+        <v>3000</v>
+      </c>
+      <c r="M39" s="48">
+        <v>50</v>
+      </c>
+      <c r="N39" s="51">
+        <v>0.65</v>
+      </c>
+      <c r="Q39" s="8">
+        <v>12</v>
+      </c>
+      <c r="R39" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="S39" s="58">
+        <v>15</v>
+      </c>
+      <c r="T39" s="57">
+        <v>0.05</v>
+      </c>
+      <c r="U39" s="30">
+        <v>20</v>
+      </c>
+      <c r="V39" s="60">
+        <v>0.2</v>
+      </c>
+      <c r="AA39" s="34">
+        <v>3000</v>
+      </c>
+      <c r="AB39" s="40">
+        <v>0.05</v>
+      </c>
+      <c r="AC39" s="44">
+        <v>1000</v>
+      </c>
+      <c r="AE39" s="51">
+        <v>0.05</v>
+      </c>
+      <c r="AF39" s="58">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A40" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B40" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C40" s="64">
+        <v>91</v>
+      </c>
+      <c r="D40" s="33">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="41" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A41" s="62" t="s">
+        <v>47</v>
+      </c>
+      <c r="B41" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="C41" s="64">
+        <v>446</v>
+      </c>
+      <c r="D41" s="33">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="42" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A42" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B42" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C42" s="64">
+        <v>174</v>
+      </c>
+      <c r="D42" s="33">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="43" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A43" s="62" t="s">
+        <v>46</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C43" s="64">
+        <v>159</v>
+      </c>
+      <c r="D43" s="33">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="44" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A44" s="62" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C44" s="64">
+        <v>155</v>
+      </c>
+      <c r="D44" s="33">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="45" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A45" s="62" t="s">
+        <v>46</v>
+      </c>
+      <c r="B45" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C45" s="64">
+        <v>241</v>
+      </c>
+      <c r="D45" s="33">
+        <v>46204</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza planilhas de controle e metadados com novas entradas e ajustes de horário. Modifica timestamps em arquivos .mtime e atualiza dados de vendedores.
</commit_message>
<xml_diff>
--- a/planilhas_cache/METAS RJ.xlsx
+++ b/planilhas_cache/METAS RJ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Drives compartilhados\Off Trade\Campanhas e Metas\METAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B55CF1-E6C1-4AB4-8314-EB94C01CE03A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40E8B484-A8FD-42CF-AAB0-3C3B4ADDD01A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{40673C59-61F7-4ACE-BE3C-88D4D3C2E782}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{40673C59-61F7-4ACE-BE3C-88D4D3C2E782}"/>
   </bookViews>
   <sheets>
     <sheet name="META_VENDEDOR" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="70">
   <si>
     <t>VENDEDOR</t>
   </si>
@@ -234,15 +234,28 @@
   </si>
   <si>
     <t>PESO POSITIVAÇÃO ESSENZA+HOB</t>
+  </si>
+  <si>
+    <t>META FATURAMENTO ESSENZA+HBO</t>
+  </si>
+  <si>
+    <t>PESO FATURAMENTO ESSENZA+HOB</t>
+  </si>
+  <si>
+    <t>META FATURAMENTO ESSENZA + HOB</t>
+  </si>
+  <si>
+    <t>PESO FATURAMENTO ESSENZA + HOB</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="169" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -604,7 +617,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="44" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -662,12 +675,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -678,9 +685,6 @@
     </xf>
     <xf numFmtId="10" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -784,6 +788,27 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1801,48 +1826,48 @@
   <dimension ref="A1:AF45"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19" style="30" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19" style="27" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.88671875" style="65" customWidth="1"/>
-    <col min="4" max="4" width="6.33203125" style="30" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.44140625" style="30" customWidth="1"/>
-    <col min="6" max="6" width="19" style="30" customWidth="1"/>
-    <col min="7" max="7" width="25.6640625" style="30" customWidth="1"/>
-    <col min="8" max="9" width="25.109375" style="30" customWidth="1"/>
-    <col min="10" max="10" width="24.5546875" style="30" customWidth="1"/>
-    <col min="11" max="11" width="28.6640625" style="30" customWidth="1"/>
-    <col min="12" max="12" width="28.109375" style="30" customWidth="1"/>
-    <col min="13" max="13" width="17.88671875" style="30" customWidth="1"/>
-    <col min="14" max="14" width="17.33203125" style="30" customWidth="1"/>
-    <col min="15" max="15" width="23.6640625" style="30" customWidth="1"/>
-    <col min="16" max="16" width="23.109375" style="30" customWidth="1"/>
-    <col min="17" max="17" width="21.5546875" style="30" customWidth="1"/>
-    <col min="18" max="18" width="21" style="30" customWidth="1"/>
-    <col min="19" max="19" width="27.33203125" style="30" customWidth="1"/>
-    <col min="20" max="20" width="26.77734375" style="30" customWidth="1"/>
-    <col min="21" max="21" width="25.6640625" style="30" customWidth="1"/>
-    <col min="22" max="22" width="25.109375" style="30" customWidth="1"/>
-    <col min="23" max="23" width="24.33203125" style="30" customWidth="1"/>
-    <col min="24" max="24" width="23.77734375" style="30" customWidth="1"/>
-    <col min="25" max="25" width="25.109375" style="30" customWidth="1"/>
-    <col min="26" max="26" width="24.5546875" style="30" customWidth="1"/>
-    <col min="27" max="27" width="28.21875" style="30" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="27.77734375" style="30" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="32.21875" style="30" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="31.77734375" style="30" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="31.33203125" style="30" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="30.88671875" style="30" bestFit="1" customWidth="1"/>
-    <col min="33" max="16384" width="8.88671875" style="30"/>
+    <col min="3" max="3" width="5.88671875" style="62" customWidth="1"/>
+    <col min="4" max="4" width="6.33203125" style="27" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.44140625" style="27" customWidth="1"/>
+    <col min="6" max="6" width="19" style="27" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" style="27" customWidth="1"/>
+    <col min="8" max="9" width="25.109375" style="27" customWidth="1"/>
+    <col min="10" max="10" width="24.5546875" style="27" customWidth="1"/>
+    <col min="11" max="11" width="28.6640625" style="27" customWidth="1"/>
+    <col min="12" max="12" width="28.109375" style="27" customWidth="1"/>
+    <col min="13" max="13" width="17.88671875" style="27" customWidth="1"/>
+    <col min="14" max="14" width="17.33203125" style="27" customWidth="1"/>
+    <col min="15" max="15" width="23.6640625" style="27" customWidth="1"/>
+    <col min="16" max="16" width="23.109375" style="27" customWidth="1"/>
+    <col min="17" max="17" width="21.5546875" style="27" customWidth="1"/>
+    <col min="18" max="18" width="21" style="27" customWidth="1"/>
+    <col min="19" max="19" width="27.33203125" style="27" customWidth="1"/>
+    <col min="20" max="20" width="26.77734375" style="27" customWidth="1"/>
+    <col min="21" max="21" width="25.6640625" style="27" customWidth="1"/>
+    <col min="22" max="22" width="25.109375" style="27" customWidth="1"/>
+    <col min="23" max="23" width="24.33203125" style="27" customWidth="1"/>
+    <col min="24" max="24" width="23.77734375" style="27" customWidth="1"/>
+    <col min="25" max="25" width="25.109375" style="27" customWidth="1"/>
+    <col min="26" max="26" width="24.5546875" style="27" customWidth="1"/>
+    <col min="27" max="27" width="28.21875" style="27" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="27.77734375" style="27" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="32.21875" style="27" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="31.77734375" style="27" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="31.33203125" style="27" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="30.88671875" style="27" bestFit="1" customWidth="1"/>
+    <col min="33" max="16384" width="8.88671875" style="27"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="58" t="s">
         <v>45</v>
       </c>
       <c r="B1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="63" t="s">
+      <c r="C1" s="60" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="11" t="s">
@@ -1914,33 +1939,33 @@
       <c r="Z1" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="AA1" s="30" t="s">
+      <c r="AA1" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="AB1" s="30" t="s">
+      <c r="AB1" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="AC1" s="30" t="s">
+      <c r="AC1" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="AD1" s="30" t="s">
+      <c r="AD1" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="AE1" s="52" t="s">
+      <c r="AE1" s="49" t="s">
         <v>64</v>
       </c>
-      <c r="AF1" s="52" t="s">
+      <c r="AF1" s="49" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:32" s="31" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="62" t="s">
+    <row r="2" spans="1:32" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="64">
+      <c r="C2" s="61">
         <v>275</v>
       </c>
       <c r="D2" s="15">
@@ -1985,14 +2010,14 @@
       <c r="Y2" s="14"/>
       <c r="Z2" s="14"/>
     </row>
-    <row r="3" spans="1:32" s="31" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+    <row r="3" spans="1:32" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="64">
+      <c r="C3" s="61">
         <v>156</v>
       </c>
       <c r="D3" s="15">
@@ -2037,14 +2062,14 @@
       <c r="Y3" s="14"/>
       <c r="Z3" s="14"/>
     </row>
-    <row r="4" spans="1:32" s="31" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="62" t="s">
+    <row r="4" spans="1:32" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="64">
+      <c r="C4" s="61">
         <v>412</v>
       </c>
       <c r="D4" s="15">
@@ -2093,14 +2118,14 @@
       <c r="Y4" s="14"/>
       <c r="Z4" s="14"/>
     </row>
-    <row r="5" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="62" t="s">
+    <row r="5" spans="1:32" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="64">
+      <c r="C5" s="61">
         <v>153</v>
       </c>
       <c r="D5" s="15">
@@ -2149,14 +2174,14 @@
       <c r="Y5" s="16"/>
       <c r="Z5" s="16"/>
     </row>
-    <row r="6" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="62" t="s">
+    <row r="6" spans="1:32" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="64">
+      <c r="C6" s="61">
         <v>158</v>
       </c>
       <c r="D6" s="15">
@@ -2201,14 +2226,14 @@
       <c r="Y6" s="16"/>
       <c r="Z6" s="16"/>
     </row>
-    <row r="7" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="62" t="s">
+    <row r="7" spans="1:32" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="64">
+      <c r="C7" s="61">
         <v>238</v>
       </c>
       <c r="D7" s="15">
@@ -2253,14 +2278,14 @@
       <c r="Y7" s="16"/>
       <c r="Z7" s="16"/>
     </row>
-    <row r="8" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="62" t="s">
+    <row r="8" spans="1:32" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="64">
+      <c r="C8" s="61">
         <v>419</v>
       </c>
       <c r="D8" s="15">
@@ -2309,14 +2334,14 @@
       <c r="Y8" s="16"/>
       <c r="Z8" s="16"/>
     </row>
-    <row r="9" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="62" t="s">
+    <row r="9" spans="1:32" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="64">
+      <c r="C9" s="61">
         <v>144</v>
       </c>
       <c r="D9" s="15">
@@ -2365,14 +2390,14 @@
       <c r="Y9" s="16"/>
       <c r="Z9" s="16"/>
     </row>
-    <row r="10" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="62" t="s">
+    <row r="10" spans="1:32" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="64">
+      <c r="C10" s="61">
         <v>450</v>
       </c>
       <c r="D10" s="15">
@@ -2417,14 +2442,14 @@
       <c r="Y10" s="16"/>
       <c r="Z10" s="16"/>
     </row>
-    <row r="11" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="62" t="s">
+    <row r="11" spans="1:32" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="59" t="s">
         <v>47</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="64">
+      <c r="C11" s="61">
         <v>417</v>
       </c>
       <c r="D11" s="15">
@@ -2473,14 +2498,14 @@
       <c r="Y11" s="16"/>
       <c r="Z11" s="16"/>
     </row>
-    <row r="12" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="62" t="s">
+    <row r="12" spans="1:32" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="59" t="s">
         <v>47</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="64">
+      <c r="C12" s="61">
         <v>439</v>
       </c>
       <c r="D12" s="15">
@@ -2529,14 +2554,14 @@
       <c r="Y12" s="16"/>
       <c r="Z12" s="16"/>
     </row>
-    <row r="13" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="62" t="s">
+    <row r="13" spans="1:32" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="59" t="s">
         <v>50</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="64">
+      <c r="C13" s="61">
         <v>420</v>
       </c>
       <c r="D13" s="15">
@@ -2573,14 +2598,14 @@
       <c r="Y13" s="16"/>
       <c r="Z13" s="16"/>
     </row>
-    <row r="14" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="62" t="s">
+    <row r="14" spans="1:32" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="59" t="s">
         <v>49</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="64">
+      <c r="C14" s="61">
         <v>431</v>
       </c>
       <c r="D14" s="15">
@@ -2641,14 +2666,14 @@
       <c r="Y14" s="16"/>
       <c r="Z14" s="16"/>
     </row>
-    <row r="15" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="62" t="s">
+    <row r="15" spans="1:32" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="59" t="s">
         <v>49</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="64">
+      <c r="C15" s="61">
         <v>379</v>
       </c>
       <c r="D15" s="15">
@@ -2709,14 +2734,14 @@
       <c r="Y15" s="16"/>
       <c r="Z15" s="16"/>
     </row>
-    <row r="16" spans="1:32" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="62" t="s">
+    <row r="16" spans="1:32" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="59" t="s">
         <v>49</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="64">
+      <c r="C16" s="61">
         <v>471</v>
       </c>
       <c r="D16" s="15">
@@ -2777,14 +2802,14 @@
       <c r="Y16" s="16"/>
       <c r="Z16" s="16"/>
     </row>
-    <row r="17" spans="1:30" s="32" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="62" t="s">
+    <row r="17" spans="1:30" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="59" t="s">
         <v>49</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="64">
+      <c r="C17" s="61">
         <v>378</v>
       </c>
       <c r="D17" s="15">
@@ -2850,13 +2875,13 @@
       <c r="Z17" s="16"/>
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A18" s="62" t="s">
+      <c r="A18" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B18" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="64">
+      <c r="C18" s="61">
         <v>91</v>
       </c>
       <c r="D18" s="15">
@@ -2886,13 +2911,13 @@
       <c r="Z18" s="13"/>
     </row>
     <row r="19" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A19" s="62" t="s">
+      <c r="A19" s="59" t="s">
         <v>47</v>
       </c>
       <c r="B19" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="64">
+      <c r="C19" s="61">
         <v>446</v>
       </c>
       <c r="D19" s="15">
@@ -2922,13 +2947,13 @@
       <c r="Z19" s="13"/>
     </row>
     <row r="20" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A20" s="62" t="s">
+      <c r="A20" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B20" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="64">
+      <c r="C20" s="61">
         <v>174</v>
       </c>
       <c r="D20" s="15">
@@ -2958,13 +2983,13 @@
       <c r="Z20" s="13"/>
     </row>
     <row r="21" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A21" s="62" t="s">
+      <c r="A21" s="59" t="s">
         <v>46</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="64">
+      <c r="C21" s="61">
         <v>159</v>
       </c>
       <c r="D21" s="15">
@@ -2994,13 +3019,13 @@
       <c r="Z21" s="13"/>
     </row>
     <row r="22" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A22" s="62" t="s">
+      <c r="A22" s="59" t="s">
         <v>46</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="64">
+      <c r="C22" s="61">
         <v>155</v>
       </c>
       <c r="D22" s="15">
@@ -3030,13 +3055,13 @@
       <c r="Z22" s="13"/>
     </row>
     <row r="23" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A23" s="62" t="s">
+      <c r="A23" s="59" t="s">
         <v>46</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="64">
+      <c r="C23" s="61">
         <v>241</v>
       </c>
       <c r="D23" s="15">
@@ -3066,531 +3091,531 @@
       <c r="Z23" s="13"/>
     </row>
     <row r="24" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="62" t="s">
+      <c r="A24" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C24" s="64">
+      <c r="C24" s="61">
         <v>275</v>
       </c>
-      <c r="D24" s="33">
+      <c r="D24" s="30">
         <v>46204</v>
       </c>
-      <c r="E24" s="34">
+      <c r="E24" s="31">
         <v>345000</v>
       </c>
-      <c r="F24" s="37">
+      <c r="F24" s="34">
         <v>0.7</v>
       </c>
-      <c r="G24" s="34">
+      <c r="G24" s="31">
         <v>44000</v>
       </c>
-      <c r="H24" s="42">
-        <v>0.1</v>
-      </c>
-      <c r="M24" s="45">
+      <c r="H24" s="39">
+        <v>0.1</v>
+      </c>
+      <c r="M24" s="42">
         <v>30</v>
       </c>
-      <c r="N24" s="49">
-        <v>0.1</v>
-      </c>
-      <c r="AA24" s="34">
+      <c r="N24" s="46">
+        <v>0.1</v>
+      </c>
+      <c r="AA24" s="31">
         <v>25000</v>
       </c>
-      <c r="AB24" s="37">
-        <v>0.05</v>
-      </c>
-      <c r="AC24" s="43">
+      <c r="AB24" s="34">
+        <v>0.05</v>
+      </c>
+      <c r="AC24" s="40">
         <v>9500</v>
       </c>
-      <c r="AD24" s="37">
+      <c r="AD24" s="34">
         <v>0.05</v>
       </c>
     </row>
     <row r="25" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="62" t="s">
+      <c r="A25" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C25" s="64">
+      <c r="C25" s="61">
         <v>156</v>
       </c>
-      <c r="D25" s="33">
+      <c r="D25" s="30">
         <v>46204</v>
       </c>
-      <c r="E25" s="34">
+      <c r="E25" s="31">
         <v>90000</v>
       </c>
-      <c r="F25" s="37">
+      <c r="F25" s="34">
         <v>0.7</v>
       </c>
-      <c r="G25" s="34">
+      <c r="G25" s="31">
         <v>9000</v>
       </c>
-      <c r="H25" s="42">
-        <v>0.1</v>
-      </c>
-      <c r="M25" s="45">
+      <c r="H25" s="39">
+        <v>0.1</v>
+      </c>
+      <c r="M25" s="42">
         <v>70</v>
       </c>
-      <c r="N25" s="49">
-        <v>0.1</v>
-      </c>
-      <c r="AA25" s="34">
+      <c r="N25" s="46">
+        <v>0.1</v>
+      </c>
+      <c r="AA25" s="31">
         <v>7000</v>
       </c>
-      <c r="AB25" s="37">
-        <v>0.05</v>
-      </c>
-      <c r="AC25" s="43">
+      <c r="AB25" s="34">
+        <v>0.05</v>
+      </c>
+      <c r="AC25" s="40">
         <v>1000</v>
       </c>
-      <c r="AD25" s="37">
+      <c r="AD25" s="34">
         <v>0.05</v>
       </c>
     </row>
     <row r="26" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="62" t="s">
+      <c r="A26" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B26" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C26" s="64">
+      <c r="C26" s="61">
         <v>412</v>
       </c>
-      <c r="D26" s="33">
+      <c r="D26" s="30">
         <v>46204</v>
       </c>
-      <c r="E26" s="34">
+      <c r="E26" s="31">
         <v>150000</v>
       </c>
-      <c r="F26" s="37">
+      <c r="F26" s="34">
         <v>0.7</v>
       </c>
-      <c r="G26" s="34">
+      <c r="G26" s="31">
         <v>9000</v>
       </c>
-      <c r="H26" s="42">
-        <v>0.1</v>
-      </c>
-      <c r="M26" s="45">
+      <c r="H26" s="39">
+        <v>0.1</v>
+      </c>
+      <c r="M26" s="42">
         <v>50</v>
       </c>
-      <c r="N26" s="49">
-        <v>0.1</v>
-      </c>
-      <c r="AA26" s="34">
+      <c r="N26" s="46">
+        <v>0.1</v>
+      </c>
+      <c r="AA26" s="31">
         <v>7000</v>
       </c>
-      <c r="AB26" s="37">
-        <v>0.05</v>
-      </c>
-      <c r="AC26" s="43">
+      <c r="AB26" s="34">
+        <v>0.05</v>
+      </c>
+      <c r="AC26" s="40">
         <v>1500</v>
       </c>
-      <c r="AD26" s="37">
+      <c r="AD26" s="34">
         <v>0.05</v>
       </c>
     </row>
     <row r="27" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="62" t="s">
+      <c r="A27" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C27" s="64">
+      <c r="C27" s="61">
         <v>153</v>
       </c>
-      <c r="D27" s="33">
+      <c r="D27" s="30">
         <v>46204</v>
       </c>
-      <c r="E27" s="34">
+      <c r="E27" s="31">
         <v>190000</v>
       </c>
-      <c r="F27" s="37">
+      <c r="F27" s="34">
         <v>0.7</v>
       </c>
-      <c r="G27" s="34">
+      <c r="G27" s="31">
         <v>10000</v>
       </c>
-      <c r="H27" s="42">
-        <v>0.1</v>
-      </c>
-      <c r="M27" s="45">
+      <c r="H27" s="39">
+        <v>0.1</v>
+      </c>
+      <c r="M27" s="42">
         <v>50</v>
       </c>
-      <c r="N27" s="49">
-        <v>0.1</v>
-      </c>
-      <c r="AA27" s="34">
+      <c r="N27" s="46">
+        <v>0.1</v>
+      </c>
+      <c r="AA27" s="31">
         <v>25000</v>
       </c>
-      <c r="AB27" s="37">
-        <v>0.05</v>
-      </c>
-      <c r="AC27" s="43">
+      <c r="AB27" s="34">
+        <v>0.05</v>
+      </c>
+      <c r="AC27" s="40">
         <v>1500</v>
       </c>
-      <c r="AD27" s="37">
+      <c r="AD27" s="34">
         <v>0.05</v>
       </c>
     </row>
     <row r="28" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="62" t="s">
+      <c r="A28" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="64">
+      <c r="C28" s="61">
         <v>158</v>
       </c>
-      <c r="D28" s="33">
+      <c r="D28" s="30">
         <v>46204</v>
       </c>
-      <c r="E28" s="34">
+      <c r="E28" s="31">
         <v>450000</v>
       </c>
-      <c r="F28" s="37">
+      <c r="F28" s="34">
         <v>0.7</v>
       </c>
-      <c r="G28" s="34">
+      <c r="G28" s="31">
         <v>12000</v>
       </c>
-      <c r="H28" s="42">
-        <v>0.1</v>
-      </c>
-      <c r="M28" s="45">
+      <c r="H28" s="39">
+        <v>0.1</v>
+      </c>
+      <c r="M28" s="42">
         <v>10</v>
       </c>
-      <c r="N28" s="49">
-        <v>0.1</v>
-      </c>
-      <c r="AA28" s="34">
+      <c r="N28" s="46">
+        <v>0.1</v>
+      </c>
+      <c r="AA28" s="31">
         <v>20000</v>
       </c>
-      <c r="AB28" s="37">
-        <v>0.05</v>
-      </c>
-      <c r="AC28" s="43">
+      <c r="AB28" s="34">
+        <v>0.05</v>
+      </c>
+      <c r="AC28" s="40">
         <v>1500</v>
       </c>
-      <c r="AD28" s="37">
+      <c r="AD28" s="34">
         <v>0.05</v>
       </c>
     </row>
     <row r="29" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="62" t="s">
+      <c r="A29" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B29" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="C29" s="64">
+      <c r="C29" s="61">
         <v>238</v>
       </c>
-      <c r="D29" s="33">
+      <c r="D29" s="30">
         <v>46204</v>
       </c>
-      <c r="E29" s="34">
+      <c r="E29" s="31">
         <v>150000</v>
       </c>
-      <c r="F29" s="37">
+      <c r="F29" s="34">
         <v>0.8</v>
       </c>
-      <c r="G29" s="34">
+      <c r="G29" s="31">
         <v>3000</v>
       </c>
-      <c r="H29" s="42">
-        <v>0.1</v>
-      </c>
-      <c r="M29" s="45">
+      <c r="H29" s="39">
+        <v>0.1</v>
+      </c>
+      <c r="M29" s="42">
         <v>1</v>
       </c>
-      <c r="N29" s="49">
-        <v>0.1</v>
-      </c>
-      <c r="AA29" s="34">
+      <c r="N29" s="46">
+        <v>0.1</v>
+      </c>
+      <c r="AA29" s="31">
         <v>0</v>
       </c>
-      <c r="AB29" s="37"/>
-      <c r="AC29" s="43">
+      <c r="AB29" s="34"/>
+      <c r="AC29" s="40">
         <v>0</v>
       </c>
-      <c r="AD29" s="37"/>
+      <c r="AD29" s="34"/>
     </row>
     <row r="30" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="62" t="s">
+      <c r="A30" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C30" s="64">
+      <c r="C30" s="61">
         <v>419</v>
       </c>
-      <c r="D30" s="33">
+      <c r="D30" s="30">
         <v>46204</v>
       </c>
-      <c r="E30" s="34">
+      <c r="E30" s="31">
         <v>130000</v>
       </c>
-      <c r="F30" s="37">
+      <c r="F30" s="34">
         <v>0.7</v>
       </c>
-      <c r="G30" s="34">
+      <c r="G30" s="31">
         <v>10000</v>
       </c>
-      <c r="H30" s="42">
-        <v>0.1</v>
-      </c>
-      <c r="M30" s="45">
+      <c r="H30" s="39">
+        <v>0.1</v>
+      </c>
+      <c r="M30" s="42">
         <v>50</v>
       </c>
-      <c r="N30" s="49">
-        <v>0.1</v>
-      </c>
-      <c r="AA30" s="34">
+      <c r="N30" s="46">
+        <v>0.1</v>
+      </c>
+      <c r="AA30" s="31">
         <v>20000</v>
       </c>
-      <c r="AB30" s="37">
-        <v>0.05</v>
-      </c>
-      <c r="AC30" s="43">
+      <c r="AB30" s="34">
+        <v>0.05</v>
+      </c>
+      <c r="AC30" s="40">
         <v>1500</v>
       </c>
-      <c r="AD30" s="37">
+      <c r="AD30" s="34">
         <v>0.05</v>
       </c>
     </row>
     <row r="31" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="62" t="s">
+      <c r="A31" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B31" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C31" s="64">
+      <c r="C31" s="61">
         <v>144</v>
       </c>
-      <c r="D31" s="33">
+      <c r="D31" s="30">
         <v>46204</v>
       </c>
-      <c r="E31" s="34">
+      <c r="E31" s="31">
         <v>190000</v>
       </c>
-      <c r="F31" s="37">
+      <c r="F31" s="34">
         <v>0.7</v>
       </c>
-      <c r="G31" s="34">
+      <c r="G31" s="31">
         <v>10000</v>
       </c>
-      <c r="H31" s="42">
-        <v>0.1</v>
-      </c>
-      <c r="M31" s="45">
+      <c r="H31" s="39">
+        <v>0.1</v>
+      </c>
+      <c r="M31" s="42">
         <v>35</v>
       </c>
-      <c r="N31" s="49">
-        <v>0.1</v>
-      </c>
-      <c r="AA31" s="34">
+      <c r="N31" s="46">
+        <v>0.1</v>
+      </c>
+      <c r="AA31" s="31">
         <v>30000</v>
       </c>
-      <c r="AB31" s="37">
-        <v>0.05</v>
-      </c>
-      <c r="AC31" s="43">
+      <c r="AB31" s="34">
+        <v>0.05</v>
+      </c>
+      <c r="AC31" s="40">
         <v>1500</v>
       </c>
-      <c r="AD31" s="37">
+      <c r="AD31" s="34">
         <v>0.05</v>
       </c>
     </row>
     <row r="32" spans="1:30" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="62" t="s">
+      <c r="A32" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B32" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C32" s="64">
+      <c r="C32" s="61">
         <v>450</v>
       </c>
-      <c r="D32" s="33">
+      <c r="D32" s="30">
         <v>46204</v>
       </c>
-      <c r="E32" s="34">
+      <c r="E32" s="31">
         <v>250000</v>
       </c>
-      <c r="F32" s="37">
+      <c r="F32" s="34">
         <v>0.7</v>
       </c>
-      <c r="G32" s="34">
+      <c r="G32" s="31">
         <v>10000</v>
       </c>
-      <c r="H32" s="42">
-        <v>0.1</v>
-      </c>
-      <c r="M32" s="45">
+      <c r="H32" s="39">
+        <v>0.1</v>
+      </c>
+      <c r="M32" s="42">
         <v>45</v>
       </c>
-      <c r="N32" s="49">
-        <v>0.1</v>
-      </c>
-      <c r="AA32" s="34">
+      <c r="N32" s="46">
+        <v>0.1</v>
+      </c>
+      <c r="AA32" s="31">
         <v>30000</v>
       </c>
-      <c r="AB32" s="37">
-        <v>0.05</v>
-      </c>
-      <c r="AC32" s="43">
+      <c r="AB32" s="34">
+        <v>0.05</v>
+      </c>
+      <c r="AC32" s="40">
         <v>1500</v>
       </c>
-      <c r="AD32" s="37">
+      <c r="AD32" s="34">
         <v>0.05</v>
       </c>
     </row>
     <row r="33" spans="1:32" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="62" t="s">
+      <c r="A33" s="59" t="s">
         <v>47</v>
       </c>
       <c r="B33" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C33" s="64">
+      <c r="C33" s="61">
         <v>439</v>
       </c>
-      <c r="D33" s="33">
+      <c r="D33" s="30">
         <v>46204</v>
       </c>
-      <c r="E33" s="34">
+      <c r="E33" s="31">
         <v>450000</v>
       </c>
-      <c r="F33" s="37">
+      <c r="F33" s="34">
         <v>0.7</v>
       </c>
-      <c r="G33" s="34">
+      <c r="G33" s="31">
         <v>10000</v>
       </c>
-      <c r="H33" s="42">
-        <v>0.1</v>
-      </c>
-      <c r="M33" s="46">
+      <c r="H33" s="39">
+        <v>0.1</v>
+      </c>
+      <c r="M33" s="43">
         <v>50</v>
       </c>
-      <c r="N33" s="49">
-        <v>0.1</v>
-      </c>
-      <c r="AA33" s="34">
+      <c r="N33" s="46">
+        <v>0.1</v>
+      </c>
+      <c r="AA33" s="31">
         <v>50000</v>
       </c>
-      <c r="AB33" s="37">
-        <v>0.05</v>
-      </c>
-      <c r="AC33" s="43">
+      <c r="AB33" s="34">
+        <v>0.05</v>
+      </c>
+      <c r="AC33" s="40">
         <v>1500</v>
       </c>
-      <c r="AD33" s="37">
+      <c r="AD33" s="34">
         <v>0.05</v>
       </c>
     </row>
     <row r="34" spans="1:32" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="62" t="s">
+      <c r="A34" s="59" t="s">
         <v>50</v>
       </c>
       <c r="B34" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C34" s="64">
+      <c r="C34" s="61">
         <v>420</v>
       </c>
-      <c r="D34" s="33">
+      <c r="D34" s="30">
         <v>46204</v>
       </c>
-      <c r="E34" s="34">
+      <c r="E34" s="31">
         <v>300000</v>
       </c>
-      <c r="F34" s="37"/>
-      <c r="G34" s="35">
+      <c r="F34" s="34"/>
+      <c r="G34" s="32">
         <v>60000</v>
       </c>
-      <c r="M34" s="45">
+      <c r="M34" s="42">
         <v>1</v>
       </c>
-      <c r="N34" s="49"/>
-      <c r="AA34" s="34">
+      <c r="N34" s="46"/>
+      <c r="AA34" s="31">
         <v>350000</v>
       </c>
-      <c r="AB34" s="37"/>
-      <c r="AC34" s="43">
+      <c r="AB34" s="34"/>
+      <c r="AC34" s="40">
         <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A35" s="62" t="s">
+      <c r="A35" s="59" t="s">
         <v>47</v>
       </c>
-      <c r="B35" s="30" t="s">
+      <c r="B35" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="C35" s="65">
+      <c r="C35" s="62">
         <v>460</v>
       </c>
-      <c r="D35" s="33">
+      <c r="D35" s="30">
         <v>46204</v>
       </c>
-      <c r="E35" s="35">
+      <c r="E35" s="32">
         <v>30000</v>
       </c>
-      <c r="F35" s="38"/>
-      <c r="G35" s="41">
+      <c r="F35" s="35"/>
+      <c r="G35" s="38">
         <v>1000</v>
       </c>
-      <c r="M35" s="45">
+      <c r="M35" s="42">
         <v>15</v>
       </c>
-      <c r="N35" s="49"/>
-      <c r="AA35" s="35">
+      <c r="N35" s="46"/>
+      <c r="AA35" s="32">
         <v>24000</v>
       </c>
-      <c r="AB35" s="38"/>
-      <c r="AC35" s="41">
+      <c r="AB35" s="35"/>
+      <c r="AC35" s="38">
         <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:32" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="62" t="s">
+      <c r="A36" s="59" t="s">
         <v>49</v>
       </c>
       <c r="B36" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C36" s="64">
+      <c r="C36" s="61">
         <v>431</v>
       </c>
-      <c r="D36" s="33">
+      <c r="D36" s="30">
         <v>46204</v>
       </c>
-      <c r="E36" s="36">
+      <c r="E36" s="33">
         <v>65000</v>
       </c>
-      <c r="F36" s="39">
-        <v>0.1</v>
-      </c>
-      <c r="G36" s="36">
+      <c r="F36" s="36">
+        <v>0.1</v>
+      </c>
+      <c r="G36" s="33">
         <v>3000</v>
       </c>
-      <c r="M36" s="47">
+      <c r="M36" s="44">
         <v>70</v>
       </c>
-      <c r="N36" s="50">
+      <c r="N36" s="47">
         <v>0.7</v>
       </c>
       <c r="Q36" s="8">
@@ -3599,54 +3624,54 @@
       <c r="R36" s="3">
         <v>0.05</v>
       </c>
-      <c r="S36" s="54">
+      <c r="S36" s="51">
         <v>15</v>
       </c>
-      <c r="T36" s="59">
-        <v>0.05</v>
-      </c>
-      <c r="AA36" s="36">
+      <c r="T36" s="56">
+        <v>0.05</v>
+      </c>
+      <c r="AA36" s="33">
         <v>3000</v>
       </c>
-      <c r="AB36" s="39">
-        <v>0.05</v>
-      </c>
-      <c r="AC36" s="44">
+      <c r="AB36" s="36">
+        <v>0.05</v>
+      </c>
+      <c r="AC36" s="41">
         <v>1000</v>
       </c>
-      <c r="AE36" s="53">
-        <v>0.05</v>
-      </c>
-      <c r="AF36" s="54">
+      <c r="AE36" s="50">
+        <v>0.05</v>
+      </c>
+      <c r="AF36" s="51">
         <v>3</v>
       </c>
     </row>
     <row r="37" spans="1:32" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="62" t="s">
+      <c r="A37" s="59" t="s">
         <v>49</v>
       </c>
       <c r="B37" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C37" s="64">
+      <c r="C37" s="61">
         <v>379</v>
       </c>
-      <c r="D37" s="33">
+      <c r="D37" s="30">
         <v>46204</v>
       </c>
-      <c r="E37" s="34">
+      <c r="E37" s="31">
         <v>80000</v>
       </c>
-      <c r="F37" s="37">
-        <v>0.1</v>
-      </c>
-      <c r="G37" s="34">
+      <c r="F37" s="34">
+        <v>0.1</v>
+      </c>
+      <c r="G37" s="31">
         <v>3000</v>
       </c>
-      <c r="M37" s="48">
+      <c r="M37" s="45">
         <v>70</v>
       </c>
-      <c r="N37" s="51">
+      <c r="N37" s="48">
         <v>0.7</v>
       </c>
       <c r="Q37" s="8">
@@ -3655,54 +3680,54 @@
       <c r="R37" s="3">
         <v>0.05</v>
       </c>
-      <c r="S37" s="58">
+      <c r="S37" s="55">
         <v>15</v>
       </c>
-      <c r="T37" s="57">
-        <v>0.05</v>
-      </c>
-      <c r="AA37" s="34">
+      <c r="T37" s="54">
+        <v>0.05</v>
+      </c>
+      <c r="AA37" s="31">
         <v>3000</v>
       </c>
-      <c r="AB37" s="37">
-        <v>0.05</v>
-      </c>
-      <c r="AC37" s="44">
+      <c r="AB37" s="34">
+        <v>0.05</v>
+      </c>
+      <c r="AC37" s="41">
         <v>1000</v>
       </c>
-      <c r="AE37" s="55">
-        <v>0.05</v>
-      </c>
-      <c r="AF37" s="56">
+      <c r="AE37" s="52">
+        <v>0.05</v>
+      </c>
+      <c r="AF37" s="53">
         <v>3</v>
       </c>
     </row>
     <row r="38" spans="1:32" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="62" t="s">
+      <c r="A38" s="59" t="s">
         <v>49</v>
       </c>
       <c r="B38" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C38" s="64">
+      <c r="C38" s="61">
         <v>471</v>
       </c>
-      <c r="D38" s="33">
+      <c r="D38" s="30">
         <v>46204</v>
       </c>
-      <c r="E38" s="34">
+      <c r="E38" s="31">
         <v>65000</v>
       </c>
-      <c r="F38" s="37">
-        <v>0.1</v>
-      </c>
-      <c r="G38" s="34">
+      <c r="F38" s="34">
+        <v>0.1</v>
+      </c>
+      <c r="G38" s="31">
         <v>3000</v>
       </c>
-      <c r="M38" s="48">
+      <c r="M38" s="45">
         <v>50</v>
       </c>
-      <c r="N38" s="51">
+      <c r="N38" s="48">
         <v>0.7</v>
       </c>
       <c r="Q38" s="8">
@@ -3711,54 +3736,54 @@
       <c r="R38" s="3">
         <v>0.05</v>
       </c>
-      <c r="S38" s="58">
+      <c r="S38" s="55">
         <v>15</v>
       </c>
-      <c r="T38" s="57">
-        <v>0.05</v>
-      </c>
-      <c r="AA38" s="34">
+      <c r="T38" s="54">
+        <v>0.05</v>
+      </c>
+      <c r="AA38" s="31">
         <v>3000</v>
       </c>
-      <c r="AB38" s="37">
-        <v>0.05</v>
-      </c>
-      <c r="AC38" s="44">
+      <c r="AB38" s="34">
+        <v>0.05</v>
+      </c>
+      <c r="AC38" s="41">
         <v>1000</v>
       </c>
-      <c r="AE38" s="57">
-        <v>0.05</v>
-      </c>
-      <c r="AF38" s="46">
+      <c r="AE38" s="54">
+        <v>0.05</v>
+      </c>
+      <c r="AF38" s="43">
         <v>3</v>
       </c>
     </row>
     <row r="39" spans="1:32" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="62" t="s">
+      <c r="A39" s="59" t="s">
         <v>49</v>
       </c>
       <c r="B39" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C39" s="64">
+      <c r="C39" s="61">
         <v>378</v>
       </c>
-      <c r="D39" s="33">
+      <c r="D39" s="30">
         <v>46204</v>
       </c>
-      <c r="E39" s="34">
+      <c r="E39" s="31">
         <v>65000</v>
       </c>
-      <c r="F39" s="40">
-        <v>0.1</v>
-      </c>
-      <c r="G39" s="34">
+      <c r="F39" s="37">
+        <v>0.1</v>
+      </c>
+      <c r="G39" s="31">
         <v>3000</v>
       </c>
-      <c r="M39" s="48">
+      <c r="M39" s="45">
         <v>50</v>
       </c>
-      <c r="N39" s="51">
+      <c r="N39" s="48">
         <v>0.65</v>
       </c>
       <c r="Q39" s="8">
@@ -3767,115 +3792,115 @@
       <c r="R39" s="3">
         <v>0.05</v>
       </c>
-      <c r="S39" s="58">
+      <c r="S39" s="55">
         <v>15</v>
       </c>
-      <c r="T39" s="57">
-        <v>0.05</v>
-      </c>
-      <c r="U39" s="30">
+      <c r="T39" s="54">
+        <v>0.05</v>
+      </c>
+      <c r="U39" s="27">
         <v>20</v>
       </c>
-      <c r="V39" s="60">
+      <c r="V39" s="57">
         <v>0.2</v>
       </c>
-      <c r="AA39" s="34">
+      <c r="AA39" s="31">
         <v>3000</v>
       </c>
-      <c r="AB39" s="40">
-        <v>0.05</v>
-      </c>
-      <c r="AC39" s="44">
+      <c r="AB39" s="37">
+        <v>0.05</v>
+      </c>
+      <c r="AC39" s="41">
         <v>1000</v>
       </c>
-      <c r="AE39" s="51">
-        <v>0.05</v>
-      </c>
-      <c r="AF39" s="58">
+      <c r="AE39" s="48">
+        <v>0.05</v>
+      </c>
+      <c r="AF39" s="55">
         <v>3</v>
       </c>
     </row>
     <row r="40" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A40" s="62" t="s">
+      <c r="A40" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B40" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="C40" s="64">
+      <c r="C40" s="61">
         <v>91</v>
       </c>
-      <c r="D40" s="33">
+      <c r="D40" s="30">
         <v>46204</v>
       </c>
     </row>
     <row r="41" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A41" s="62" t="s">
+      <c r="A41" s="59" t="s">
         <v>47</v>
       </c>
       <c r="B41" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="C41" s="64">
+      <c r="C41" s="61">
         <v>446</v>
       </c>
-      <c r="D41" s="33">
+      <c r="D41" s="30">
         <v>46204</v>
       </c>
     </row>
     <row r="42" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A42" s="62" t="s">
+      <c r="A42" s="59" t="s">
         <v>48</v>
       </c>
       <c r="B42" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C42" s="64">
+      <c r="C42" s="61">
         <v>174</v>
       </c>
-      <c r="D42" s="33">
+      <c r="D42" s="30">
         <v>46204</v>
       </c>
     </row>
     <row r="43" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A43" s="62" t="s">
+      <c r="A43" s="59" t="s">
         <v>46</v>
       </c>
       <c r="B43" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C43" s="64">
+      <c r="C43" s="61">
         <v>159</v>
       </c>
-      <c r="D43" s="33">
+      <c r="D43" s="30">
         <v>46204</v>
       </c>
     </row>
     <row r="44" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A44" s="62" t="s">
+      <c r="A44" s="59" t="s">
         <v>46</v>
       </c>
       <c r="B44" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C44" s="64">
+      <c r="C44" s="61">
         <v>155</v>
       </c>
-      <c r="D44" s="33">
+      <c r="D44" s="30">
         <v>46204</v>
       </c>
     </row>
     <row r="45" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A45" s="62" t="s">
+      <c r="A45" s="59" t="s">
         <v>46</v>
       </c>
       <c r="B45" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C45" s="64">
+      <c r="C45" s="61">
         <v>241</v>
       </c>
-      <c r="D45" s="33">
+      <c r="D45" s="30">
         <v>46204</v>
       </c>
     </row>
@@ -3890,29 +3915,32 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{650E0CD0-BD77-4589-B149-C9A38D814DA1}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15" style="31" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25" style="31" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17" style="31" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="24.44140625" style="31" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="24" style="31" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="30"/>
+    <col min="1" max="1" width="10.6640625" style="28" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" style="28" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5546875" style="28" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" style="28" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.5546875" style="65" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.109375" style="28" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25" style="28" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.5546875" style="28" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17" style="28" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.5546875" style="28" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.44140625" style="28" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="24" style="28" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="30.21875" style="65" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="29.6640625" style="28" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.44140625" style="65" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.88671875" style="28"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A1" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="19" t="s">
         <v>52</v>
       </c>
       <c r="C1" s="19" t="s">
@@ -3921,7 +3949,7 @@
       <c r="D1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="63" t="s">
         <v>28</v>
       </c>
       <c r="F1" s="20" t="s">
@@ -3945,12 +3973,21 @@
       <c r="L1" s="20" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="22" t="s">
+      <c r="M1" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="N1" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="O1" s="20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="14" t="s">
         <v>58</v>
       </c>
       <c r="C2" s="14">
@@ -3959,7 +3996,7 @@
       <c r="D2" s="21">
         <v>46174</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="64">
         <v>3300000</v>
       </c>
       <c r="F2" s="3">
@@ -3982,6 +4019,52 @@
       </c>
       <c r="L2" s="3">
         <v>0.05</v>
+      </c>
+      <c r="M2" s="66"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="66"/>
+    </row>
+    <row r="3" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="14">
+        <v>238</v>
+      </c>
+      <c r="D3" s="21">
+        <v>46204</v>
+      </c>
+      <c r="E3" s="67">
+        <v>3000000</v>
+      </c>
+      <c r="F3" s="68">
+        <v>0.7</v>
+      </c>
+      <c r="G3" s="2">
+        <v>200000</v>
+      </c>
+      <c r="H3" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="I3" s="14">
+        <v>600</v>
+      </c>
+      <c r="J3" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="66">
+        <v>25000</v>
+      </c>
+      <c r="N3" s="14">
+        <v>15</v>
+      </c>
+      <c r="O3" s="66">
+        <v>600000</v>
       </c>
     </row>
   </sheetData>
@@ -3991,35 +4074,37 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4055FAD4-CB0B-425C-885A-453CFD64A59E}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.5546875" style="30" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" style="30" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.33203125" style="30" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" style="30" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" style="30" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.77734375" style="30" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.77734375" style="30" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.21875" style="30" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.5546875" style="30" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16" style="30" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="24" style="30" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.44140625" style="30" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="30"/>
+    <col min="1" max="1" width="9.5546875" style="27" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" style="27" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.33203125" style="27" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" style="27" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.33203125" style="27" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.77734375" style="27" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.77734375" style="27" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.21875" style="27" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.5546875" style="27" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16" style="27" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24" style="27" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.44140625" style="27" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.77734375" style="27" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="31.5546875" style="27" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.88671875" style="27"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="C1" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="29" t="s">
+      <c r="D1" s="26" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="20" t="s">
@@ -4046,43 +4131,91 @@
       <c r="L1" s="20" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="23" t="s">
+      <c r="M1" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="N1" s="20" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="24">
+      <c r="C2" s="22">
         <v>6</v>
       </c>
-      <c r="D2" s="25">
+      <c r="D2" s="23">
         <v>46174</v>
       </c>
-      <c r="E2" s="26">
+      <c r="E2" s="24">
         <v>3300000</v>
       </c>
-      <c r="F2" s="27">
+      <c r="F2" s="25">
         <v>0.75</v>
       </c>
-      <c r="G2" s="26">
+      <c r="G2" s="24">
         <v>200000</v>
       </c>
-      <c r="H2" s="27">
-        <v>0.05</v>
-      </c>
-      <c r="I2" s="24">
+      <c r="H2" s="25">
+        <v>0.05</v>
+      </c>
+      <c r="I2" s="22">
         <v>600</v>
       </c>
-      <c r="J2" s="27">
+      <c r="J2" s="25">
         <v>0.15</v>
       </c>
-      <c r="K2" s="24">
+      <c r="K2" s="22">
         <v>30</v>
       </c>
-      <c r="L2" s="27">
-        <v>0.05</v>
+      <c r="L2" s="25">
+        <v>0.05</v>
+      </c>
+      <c r="M2" s="24"/>
+      <c r="N2" s="22"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="22">
+        <v>6</v>
+      </c>
+      <c r="D3" s="23">
+        <v>46204</v>
+      </c>
+      <c r="E3" s="24">
+        <v>3300000</v>
+      </c>
+      <c r="F3" s="25">
+        <v>0.7</v>
+      </c>
+      <c r="G3" s="24">
+        <v>200000</v>
+      </c>
+      <c r="H3" s="25">
+        <v>0.05</v>
+      </c>
+      <c r="I3" s="22">
+        <v>600</v>
+      </c>
+      <c r="J3" s="25">
+        <v>0.1</v>
+      </c>
+      <c r="K3" s="22"/>
+      <c r="L3" s="25"/>
+      <c r="M3" s="24">
+        <v>25000</v>
+      </c>
+      <c r="N3" s="69">
+        <v>0.15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>